<commit_message>
Add cross-foot and range-length checks, fix audit gaps, add tests/CI
Implement CROSS_FOOT_FAILURE and RANGE_LENGTH_MISMATCH checks and wire up materiality, headline outputs, and range-expansion config. Fix reference out-of-range false positives, year-literal noise, annotation of range/multi-cell findings, exit-code semantics (add --strict), and the config rule-id mapping.

Add pytest suite (unit, corpus, schema, exit-code), requirements files, and CI workflow with LibreOffice. Add project logo and SEO-focused README, trim unimplemented rules from docs, and stop tracking generated dist/ artifacts.
</commit_message>
<xml_diff>
--- a/assets/test_corpus/seeded_defects/seeded-defects.xlsx
+++ b/assets/test_corpus/seeded_defects/seeded-defects.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:F70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -767,6 +767,129 @@
       </c>
       <c r="B44" t="e">
         <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Range length mismatch block</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="F60">
+        <f>SUM(B60:D60)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="F61">
+        <f>SUM(C61:E61)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="F62">
+        <f>SUM(B62:D62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="F63">
+        <f>SUM(B63:C63)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Cross-foot block</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>10</v>
+      </c>
+      <c r="C68" t="n">
+        <v>20</v>
+      </c>
+      <c r="D68" t="n">
+        <v>30</v>
+      </c>
+      <c r="E68">
+        <f>SUM(B68:D68)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>5</v>
+      </c>
+      <c r="C69" t="n">
+        <v>15</v>
+      </c>
+      <c r="D69" t="n">
+        <v>25</v>
+      </c>
+      <c r="E69">
+        <f>SUM(B69:D69)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B70">
+        <f>SUM(B68:B68)</f>
+        <v/>
+      </c>
+      <c r="C70">
+        <f>SUM(C68:C69)</f>
+        <v/>
+      </c>
+      <c r="D70">
+        <f>SUM(D68:D69)</f>
+        <v/>
+      </c>
+      <c r="E70">
+        <f>SUM(E68:E69)</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>